<commit_message>
Separa finanzas personales y WEIT en dos archivos
Personal: ingresos Tiburones + salario WEIT, sin operación de WEIT (7 bolsillos).
WEIT: ingresos variables (promedio 5.000.000), operación y salario del dueño (4 bolsillos).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrxwGH7E6q3Koytg9qgEq2
</commit_message>
<xml_diff>
--- a/Finanzas_Personales.xlsx
+++ b/Finanzas_Personales.xlsx
@@ -21,13 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="$#,##0;[Red]-$#,##0;-"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="mmmm yyyy"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="169" formatCode="mmm yyyy"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -36,10 +37,6 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -56,6 +53,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
@@ -131,45 +132,45 @@
   </cellStyleXfs>
   <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -708,7 +709,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. Hoja Plan: revisa que ingresos y gastos estén bien y anota en 'Saldo inicial' lo que ya tienes en cada bolsillo. Solo se hace una vez.</t>
+          <t>1. Hoja Plan: revisa ingresos y gastos y anota en 'Saldo inicial' lo que ya tienes en cada bolsillo. Solo se hace una vez.</t>
         </is>
       </c>
     </row>
@@ -739,14 +740,14 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>LOS 8 BOLSILLOS</t>
+          <t>LOS 7 BOLSILLOS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Fijos del mes · Deudas y apartamento · WEIT operación · Mis gastos · Viajes y regalos · Emergencias y carro · Inversión sueños · Colchón WEIT</t>
+          <t>Fijos del mes · Deudas y apartamento · Mis gastos · Viajes y regalos · Emergencias y carro · Inversión sueños · Colchón personal</t>
         </is>
       </c>
     </row>
@@ -763,28 +764,28 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>RUTINA DE DÍA DE PAGO</t>
+          <t>REGLA CLAVE</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Al recibir Tiburones: transfiere a cada bolsillo su plan mensual (mira la hoja Resumen).</t>
+          <t>Tus ingresos personales son solo dos: Club Tiburones y el salario fijo que WEIT te paga. Todo lo demás que gane WEIT se queda en el archivo de WEIT.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Al recibir pagos de WEIT: primero WEIT operación, luego Deudas y apartamento, y lo que sobre va al Colchón.</t>
+          <t>Cuando WEIT te transfiera el salario, anótalo aquí como Ingreso (fuente 'Salario WEIT').</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Una vez al mes: compara el 'Saldo acumulado' de la hoja Resumen con el saldo real de cada bolsillo. Deben coincidir.</t>
+          <t>Una vez al mes compara el 'Saldo acumulado' del Resumen con el saldo real de cada bolsillo. Deben coincidir.</t>
         </is>
       </c>
     </row>
@@ -826,21 +827,21 @@
     <col width="3" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan mensual</t>
+          <t>Plan mensual – Finanzas personales</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Celdas azules con fondo amarillo = las que tú editas. Todo en pesos COP completos (4.200.000, no 4.200). Fuente de los montos: los que me diste en la conversación.</t>
+          <t>Celdas azules con fondo amarillo = las que tú editas. Todo en pesos COP completos (4.200.000, no 4.200). Montos: los que diste en la conversación. WEIT solo entra por tu salario fijo; la operación de WEIT va en su propio archivo.</t>
         </is>
       </c>
     </row>
@@ -853,7 +854,7 @@
       <c r="B4" s="6" t="n"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>BOLSILLOS (8 en total)</t>
+          <t>BOLSILLOS (7 en total)</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
@@ -893,11 +894,11 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>WEIT – entrenamientos personalizados (promedio)</t>
+          <t>Salario que te paga WEIT (fijo, como trabajador)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>4000000</v>
+        <v>2710000</v>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
@@ -924,7 +925,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>B5+B6</f>
+        <f>SUM(B5:B6)</f>
         <v/>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -956,12 +957,12 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>WEIT operación</t>
+          <t>Mis gastos</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Kelly, transporte y entrenadores auxiliares</t>
+          <t>Tu plata personal para gastar sin culpa</t>
         </is>
       </c>
       <c r="H8" s="12">
@@ -975,12 +976,12 @@
     <row r="9" ht="28" customHeight="1">
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Mis gastos</t>
+          <t>Viajes y regalos</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Tu plata personal para gastar sin culpa</t>
+          <t>Viajes y cumpleaños: se acumula entre meses</t>
         </is>
       </c>
       <c r="H9" s="12">
@@ -1002,12 +1003,12 @@
       <c r="D10" s="6" t="n"/>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Viajes y regalos</t>
+          <t>Emergencias y carro</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Viajes y cumpleaños: se acumula entre meses</t>
+          <t>Fondo de emergencia + imprevistos del carro</t>
         </is>
       </c>
       <c r="H10" s="12">
@@ -1041,12 +1042,12 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Emergencias y carro</t>
+          <t>Inversión sueños</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Fondo de emergencia + imprevistos del carro</t>
+          <t>Ahorro/inversión para tus metas</t>
         </is>
       </c>
       <c r="H11" s="12">
@@ -1076,25 +1077,25 @@
       <c r="D12" s="8" t="n">
         <v>400000</v>
       </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Inversión sueños</t>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Colchón personal</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Ahorro/inversión para tus metas</t>
+          <t>Lo que sobra cada mes: impuestos, imprevistos o para adelantar deudas</t>
         </is>
       </c>
       <c r="H12" s="12">
-        <f>SUMIFS($D$12:$D$41,$B$12:$B$41,F12)</f>
+        <f>B7-SUM(H6:H11)</f>
         <v/>
       </c>
       <c r="I12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Seguro apto</t>
@@ -1113,22 +1114,19 @@
       <c r="D13" s="8" t="n">
         <v>46000</v>
       </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>Colchón WEIT</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>Lo que sobra cada mes. Cubre los meses en que WEIT entra por debajo del promedio</t>
-        </is>
-      </c>
-      <c r="H13" s="12">
-        <f>B7-SUM(H6:H12)</f>
-        <v/>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0</v>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="14">
+        <f>SUM(H6:H12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="14">
+        <f>SUM(I6:I12)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1150,19 +1148,10 @@
       <c r="D14" s="8" t="n">
         <v>24000</v>
       </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="14">
-        <f>SUM(H6:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="14">
-        <f>SUM(I6:I13)</f>
-        <v/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Saldo inicial = lo que ya tienes guardado hoy en cada bolsillo. El último bolsillo se calcula solo: ingresos − los otros 6.</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1184,11 +1173,6 @@
       <c r="D15" s="8" t="n">
         <v>40000</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Saldo inicial = lo que ya tienes guardado hoy en cada bolsillo. El Colchón se calcula solo: ingresos − los otros 7 bolsillos.</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1209,6 +1193,14 @@
       <c r="D16" s="8" t="n">
         <v>20000</v>
       </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>CUADRE POR FUENTE DE INGRESO</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -1229,14 +1221,26 @@
       <c r="D17" s="8" t="n">
         <v>160000</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>CUADRE POR FUENTE DE INGRESO</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Ingreso esperado</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Gastos que paga</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Sobra / (falta)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -1257,25 +1261,22 @@
       <c r="D18" s="8" t="n">
         <v>210000</v>
       </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>Ingreso esperado</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Gastos que paga</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>Sobra / (falta)</t>
-        </is>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Club Tiburones</t>
+        </is>
+      </c>
+      <c r="G18" s="12">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="H18" s="12">
+        <f>SUMIFS($D$12:$D$41,$C$12:$C$41,F18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="18">
+        <f>G18-H18</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1299,11 +1300,11 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Club Tiburones</t>
+          <t>Salario WEIT</t>
         </is>
       </c>
       <c r="G19" s="12">
-        <f>B5</f>
+        <f>B6</f>
         <v/>
       </c>
       <c r="H19" s="12">
@@ -1328,27 +1329,27 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Salario WEIT</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
         <v>2110000</v>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>WEIT</t>
-        </is>
-      </c>
-      <c r="G20" s="12">
-        <f>B6</f>
-        <v/>
-      </c>
-      <c r="H20" s="12">
-        <f>SUMIFS($D$12:$D$41,$C$12:$C$41,F20)</f>
-        <v/>
-      </c>
-      <c r="I20" s="18">
-        <f>G20-H20</f>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G20" s="14">
+        <f>SUM(G18:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="14">
+        <f>SUM(H18:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="14">
+        <f>SUM(I18:I19)</f>
         <v/>
       </c>
     </row>
@@ -1365,28 +1366,16 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Salario WEIT</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
         <v>600000</v>
       </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="G21" s="14">
-        <f>SUM(G19:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="14">
-        <f>SUM(H19:H20)</f>
-        <v/>
-      </c>
-      <c r="I21" s="14">
-        <f>SUM(I19:I20)</f>
-        <v/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>El salario de WEIT cubre el apartamento; Tiburones cubre el resto y lo que sobra va al Colchón.</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1408,11 +1397,6 @@
       <c r="D22" s="8" t="n">
         <v>500000</v>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Si WEIT sale en negativo, lo cubre el sobrante de Tiburones (esa es la lógica del Colchón).</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -1433,112 +1417,126 @@
       <c r="D23" s="8" t="n">
         <v>250000</v>
       </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>INDICADORES</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>Mis gastos personales</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>WEIT operación</t>
+          <t>Mis gastos</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Club Tiburones</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>INDICADORES</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
+        <v>600000</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Deudas y apartamento / ingreso</t>
+        </is>
+      </c>
+      <c r="G24" s="19">
+        <f>IF(B7=0,0,H7/B7)</f>
+        <v/>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Sana: menos de 35%</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Transporte</t>
+          <t>Viajes</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>WEIT operación</t>
+          <t>Viajes y regalos</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Club Tiburones</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>600000</v>
+        <v>200000</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Deudas y apartamento / ingreso</t>
+          <t>Ahorro (emergencias + sueños + colchón) / ingreso</t>
         </is>
       </c>
       <c r="G25" s="19">
-        <f>IF(B7=0,0,H7/B7)</f>
+        <f>IF(B7=0,0,(H10+H11+H12)/B7)</f>
         <v/>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Sana: menos de 35%</t>
+          <t>Meta: 15–20%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Entrenadores auxiliares</t>
+          <t>Cumpleaños familia y allegados</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>WEIT operación</t>
+          <t>Viajes y regalos</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Club Tiburones</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>250000</v>
+        <v>350000</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Ahorro (emergencias + sueños + colchón) / ingreso</t>
-        </is>
-      </c>
-      <c r="G26" s="19">
-        <f>IF(B7=0,0,(H11+H12+H13)/B7)</f>
+          <t>Meta fondo de emergencia (6 meses de gastos)</t>
+        </is>
+      </c>
+      <c r="G26" s="12">
+        <f>6*SUM(H6:H11)</f>
         <v/>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Meta: 15–20%</t>
+          <t>Meta a largo plazo</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Mis gastos personales</t>
+          <t>Imprevistos carro</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Mis gastos</t>
+          <t>Emergencias y carro</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -1547,32 +1545,18 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>600000</v>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Meta fondo de emergencia (6 meses de gastos)</t>
-        </is>
-      </c>
-      <c r="G27" s="12">
-        <f>6*SUM(H6:H12)</f>
-        <v/>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Ingreso variable = 6 meses</t>
-        </is>
+        <v>200000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Fondo de emergencia</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Viajes y regalos</t>
+          <t>Emergencias y carro</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1587,12 +1571,12 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Cumpleaños familia y allegados</t>
+          <t>Inversión sueños</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Viajes y regalos</t>
+          <t>Inversión sueños</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -1601,68 +1585,26 @@
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>350000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>Imprevistos carro</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Emergencias y carro</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Club Tiburones</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Fondo de emergencia</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Emergencias y carro</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Club Tiburones</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Inversión sueños</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Inversión sueños</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>Club Tiburones</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -1734,17 +1676,17 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Tienes filas libres hasta la 41 para agregar gastos nuevos: elige su bolsillo en la lista.</t>
+          <t>Hay filas libres hasta la 41 para agregar gastos nuevos: elige su bolsillo en la lista.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B12:B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=$F$6:$F$13</formula1>
+      <formula1>=$F$6:$F$12</formula1>
     </dataValidation>
     <dataValidation sqref="C12:C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Club Tiburones,WEIT"</formula1>
+      <formula1>"Club Tiburones,Salario WEIT"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1785,7 +1727,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Las 3 filas de ejemplo (dice 'ejemplo') son solo para mostrar el formato: bórralas cuando empieces.</t>
+          <t>Las filas de ejemplo (dicen 'ejemplo') son solo para mostrar el formato: bórralas cuando empieces.</t>
         </is>
       </c>
     </row>
@@ -1850,25 +1792,25 @@
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>Gasto</t>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>Spotify (ejemplo)</t>
+          <t>Salario WEIT (ejemplo)</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Fijos del mes</t>
+          <t>Salario WEIT</t>
         </is>
       </c>
       <c r="E7" s="22" t="n">
-        <v>24000</v>
+        <v>2710000</v>
       </c>
       <c r="F7" s="23">
         <f>IF(A7="","",DATE(YEAR(A7),MONTH(A7),1))</f>
@@ -1877,7 +1819,7 @@
     </row>
     <row r="8">
       <c r="A8" s="20" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
@@ -1886,16 +1828,16 @@
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>Almuerzo con amigos (ejemplo)</t>
+          <t>Spotify (ejemplo)</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Mis gastos</t>
+          <t>Fijos del mes</t>
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>65000</v>
+        <v>24000</v>
       </c>
       <c r="F8" s="23">
         <f>IF(A8="","",DATE(YEAR(A8),MONTH(A8),1))</f>
@@ -1903,11 +1845,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="22" t="n"/>
+      <c r="A9" s="20" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Almuerzo con amigos (ejemplo)</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Mis gastos</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>65000</v>
+      </c>
       <c r="F9" s="23">
         <f>IF(A9="","",DATE(YEAR(A9),MONTH(A9),1))</f>
         <v/>
@@ -7375,7 +7333,7 @@
       <formula1>"Ingreso,Gasto"</formula1>
     </dataValidation>
     <dataValidation sqref="D6:D505" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Listas!$A$2:$A$11</formula1>
+      <formula1>=Listas!$A$2:$A$10</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7388,10 +7346,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -7492,7 +7450,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>WEIT</t>
+          <t>Salario WEIT</t>
         </is>
       </c>
       <c r="B10" s="27">
@@ -7754,8 +7712,8 @@
         <f>Plan!F12</f>
         <v/>
       </c>
-      <c r="B24" s="27">
-        <f>Plan!H12</f>
+      <c r="B24" s="12">
+        <f>IF($C$11&gt;0,$C$11,$B$11)-SUM(B18:B23)</f>
         <v/>
       </c>
       <c r="C24" s="27">
@@ -7767,7 +7725,7 @@
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>Plan!I12+Plan!H12*$B$5-SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Gasto",Movimientos!$D$6:$D$505,$A24,Movimientos!$F$6:$F$505,"&lt;="&amp;$B$4,Movimientos!$F$6:$F$505,"&gt;="&amp;Plan!$B$8)</f>
+        <f>Plan!I12+SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Ingreso",Movimientos!$F$6:$F$505,"&lt;="&amp;$B$4,Movimientos!$F$6:$F$505,"&gt;="&amp;Plan!$B$8)-SUM(Plan!$H$6:$H$11)*$B$5-SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Gasto",Movimientos!$D$6:$D$505,$A24,Movimientos!$F$6:$F$505,"&lt;="&amp;$B$4,Movimientos!$F$6:$F$505,"&gt;="&amp;Plan!$B$8)</f>
         <v/>
       </c>
       <c r="F24" s="7">
@@ -7776,64 +7734,49 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28">
-        <f>Plan!F13</f>
-        <v/>
-      </c>
-      <c r="B25" s="12">
-        <f>IF($C$11&gt;0,$C$11,$B$11)-SUM(B18:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="27">
-        <f>SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Gasto",Movimientos!$D$6:$D$505,$A25,Movimientos!$F$6:$F$505,$B$4)</f>
-        <v/>
-      </c>
-      <c r="D25" s="12">
-        <f>B25-C25</f>
-        <v/>
-      </c>
-      <c r="E25" s="12">
-        <f>Plan!I13+SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Ingreso",Movimientos!$F$6:$F$505,"&lt;="&amp;$B$4,Movimientos!$F$6:$F$505,"&gt;="&amp;Plan!$B$8)-SUM(Plan!$H$6:$H$12)*$B$5-SUMIFS(Movimientos!$E$6:$E$505,Movimientos!$B$6:$B$505,"Gasto",Movimientos!$D$6:$D$505,$A25,Movimientos!$F$6:$F$505,"&lt;="&amp;$B$4,Movimientos!$F$6:$F$505,"&gt;="&amp;Plan!$B$8)</f>
-        <v/>
-      </c>
-      <c r="F25" s="7">
-        <f>IF(E25&lt;0,"Saldo negativo",IF(D25&lt;0,"Gastaste más del plan","OK"))</f>
-        <v/>
-      </c>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B25" s="14">
+        <f>SUM(B18:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="14">
+        <f>SUM(C18:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="14">
+        <f>SUM(D18:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="14">
+        <f>SUM(E18:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="17" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B26" s="14">
-        <f>SUM(B18:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="14">
-        <f>SUM(C18:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="14">
-        <f>SUM(D18:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="14">
-        <f>SUM(E18:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="17" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Colchón WEIT: su 'Plan del mes' es lo que realmente sobró (ingreso real − los otros 7 bolsillos). Si WEIT entra bajo, este número baja y el saldo acumulado te dice cuánto respaldo tienes.</t>
-        </is>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Colchón: su 'Plan del mes' es lo que realmente sobró (ingreso real − los otros bolsillos). No cuentes con dinero de WEIT aparte de tu salario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Meses de gastos que cubre el último bolsillo (colchón)</t>
+        </is>
+      </c>
+      <c r="B28" s="29">
+        <f>IF(SUM(B18:B23)=0,0,E24/SUM(B18:B23))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F18:F25">
+  <conditionalFormatting sqref="F18:F24">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F18&lt;&gt;"OK"</formula>
     </cfRule>
@@ -7878,12 +7821,12 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ingreso Tiburones</t>
+          <t>Ingreso Club Tiburones</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Ingreso WEIT</t>
+          <t>Ingreso Salario WEIT</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -7908,7 +7851,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29">
+      <c r="A5" s="30">
         <f>Plan!B8</f>
         <v/>
       </c>
@@ -7921,7 +7864,7 @@
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>B5+C5</f>
+        <f>SUM(B5:C5)</f>
         <v/>
       </c>
       <c r="E5" s="27">
@@ -7938,7 +7881,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30">
+      <c r="A6" s="31">
         <f>EDATE(A5,1)</f>
         <v/>
       </c>
@@ -7951,7 +7894,7 @@
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>B6+C6</f>
+        <f>SUM(B6:C6)</f>
         <v/>
       </c>
       <c r="E6" s="27">
@@ -7968,7 +7911,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30">
+      <c r="A7" s="31">
         <f>EDATE(A6,1)</f>
         <v/>
       </c>
@@ -7981,7 +7924,7 @@
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>B7+C7</f>
+        <f>SUM(B7:C7)</f>
         <v/>
       </c>
       <c r="E7" s="27">
@@ -7998,7 +7941,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30">
+      <c r="A8" s="31">
         <f>EDATE(A7,1)</f>
         <v/>
       </c>
@@ -8011,7 +7954,7 @@
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>B8+C8</f>
+        <f>SUM(B8:C8)</f>
         <v/>
       </c>
       <c r="E8" s="27">
@@ -8028,7 +7971,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30">
+      <c r="A9" s="31">
         <f>EDATE(A8,1)</f>
         <v/>
       </c>
@@ -8041,7 +7984,7 @@
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>B9+C9</f>
+        <f>SUM(B9:C9)</f>
         <v/>
       </c>
       <c r="E9" s="27">
@@ -8058,7 +8001,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30">
+      <c r="A10" s="31">
         <f>EDATE(A9,1)</f>
         <v/>
       </c>
@@ -8071,7 +8014,7 @@
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>B10+C10</f>
+        <f>SUM(B10:C10)</f>
         <v/>
       </c>
       <c r="E10" s="27">
@@ -8088,7 +8031,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30">
+      <c r="A11" s="31">
         <f>EDATE(A10,1)</f>
         <v/>
       </c>
@@ -8101,7 +8044,7 @@
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>B11+C11</f>
+        <f>SUM(B11:C11)</f>
         <v/>
       </c>
       <c r="E11" s="27">
@@ -8118,7 +8061,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30">
+      <c r="A12" s="31">
         <f>EDATE(A11,1)</f>
         <v/>
       </c>
@@ -8131,7 +8074,7 @@
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>B12+C12</f>
+        <f>SUM(B12:C12)</f>
         <v/>
       </c>
       <c r="E12" s="27">
@@ -8148,7 +8091,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30">
+      <c r="A13" s="31">
         <f>EDATE(A12,1)</f>
         <v/>
       </c>
@@ -8161,7 +8104,7 @@
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>B13+C13</f>
+        <f>SUM(B13:C13)</f>
         <v/>
       </c>
       <c r="E13" s="27">
@@ -8178,7 +8121,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30">
+      <c r="A14" s="31">
         <f>EDATE(A13,1)</f>
         <v/>
       </c>
@@ -8191,7 +8134,7 @@
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>B14+C14</f>
+        <f>SUM(B14:C14)</f>
         <v/>
       </c>
       <c r="E14" s="27">
@@ -8208,7 +8151,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30">
+      <c r="A15" s="31">
         <f>EDATE(A14,1)</f>
         <v/>
       </c>
@@ -8221,7 +8164,7 @@
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>B15+C15</f>
+        <f>SUM(B15:C15)</f>
         <v/>
       </c>
       <c r="E15" s="27">
@@ -8238,7 +8181,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30">
+      <c r="A16" s="31">
         <f>EDATE(A15,1)</f>
         <v/>
       </c>
@@ -8251,7 +8194,7 @@
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>B16+C16</f>
+        <f>SUM(B16:C16)</f>
         <v/>
       </c>
       <c r="E16" s="27">
@@ -8307,78 +8250,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="31" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Lista para el desplegable de Movimientos (no editar)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Club Tiburones</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="31" t="inlineStr">
-        <is>
-          <t>WEIT</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Salario WEIT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="31">
+      <c r="A4">
         <f>Plan!F6</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="31">
+      <c r="A5">
         <f>Plan!F7</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31">
+      <c r="A6">
         <f>Plan!F8</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31">
+      <c r="A7">
         <f>Plan!F9</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="31">
+      <c r="A8">
         <f>Plan!F10</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31">
+      <c r="A9">
         <f>Plan!F11</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31">
+      <c r="A10">
         <f>Plan!F12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="31">
-        <f>Plan!F13</f>
         <v/>
       </c>
     </row>

</xml_diff>